<commit_message>
implement Appeal Chance live & improved txt line read
</commit_message>
<xml_diff>
--- a/sdk/Skill Effect.xlsx
+++ b/sdk/Skill Effect.xlsx
@@ -500,7 +500,7 @@
     <t xml:space="preserve">AddCollaboGaugeGimmickBuff  </t>
   </si>
   <si>
-    <t>LiveBuff (5)</t>
+    <t>ActiveBuffNonCleanse (5)</t>
   </si>
   <si>
     <t xml:space="preserve">AddCriticalRateGimmickBuff  </t>
@@ -662,7 +662,7 @@
     <t xml:space="preserve">AddActionSkillRateLiveDebuff  </t>
   </si>
   <si>
-    <t>LiveDebuff (6)</t>
+    <t>ActiveDebuffNonCleanse (6)</t>
   </si>
   <si>
     <t>Base Voltage Down</t>
@@ -2828,7 +2828,7 @@
     <col min="2" max="2" width="74.5714285714286" customWidth="1"/>
     <col min="3" max="3" width="59.4285714285714" customWidth="1"/>
     <col min="4" max="4" width="52.8571428571429" customWidth="1"/>
-    <col min="5" max="5" width="26" style="2" customWidth="1"/>
+    <col min="5" max="5" width="28.7142857142857" style="2" customWidth="1"/>
     <col min="6" max="6" width="30.5714285714286" style="2" customWidth="1"/>
     <col min="7" max="7" width="14.8571428571429" customWidth="1"/>
     <col min="8" max="8" width="7.57142857142857" style="2" customWidth="1"/>
@@ -5171,7 +5171,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="79" hidden="1" spans="1:10">
+    <row r="79" ht="27" hidden="1" spans="1:10">
       <c r="A79" s="3">
         <v>78</v>
       </c>
@@ -5199,7 +5199,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="80" hidden="1" spans="1:10">
+    <row r="80" ht="27" hidden="1" spans="1:10">
       <c r="A80" s="3">
         <v>79</v>
       </c>
@@ -5227,7 +5227,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="81" hidden="1" spans="1:10">
+    <row r="81" ht="27" hidden="1" spans="1:10">
       <c r="A81" s="3">
         <v>80</v>
       </c>
@@ -5255,7 +5255,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="82" hidden="1" spans="1:10">
+    <row r="82" ht="27" hidden="1" spans="1:10">
       <c r="A82" s="3">
         <v>81</v>
       </c>
@@ -5283,7 +5283,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="83" hidden="1" spans="1:10">
+    <row r="83" ht="27" hidden="1" spans="1:10">
       <c r="A83" s="3">
         <v>82</v>
       </c>
@@ -5311,7 +5311,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="84" hidden="1" spans="1:10">
+    <row r="84" ht="27" hidden="1" spans="1:10">
       <c r="A84" s="3">
         <v>83</v>
       </c>
@@ -5989,7 +5989,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="106" hidden="1" spans="1:10">
+    <row r="106" ht="27" hidden="1" spans="1:10">
       <c r="A106" s="3">
         <v>105</v>
       </c>
@@ -6911,7 +6911,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="136" hidden="1" spans="1:10">
+    <row r="136" ht="27" hidden="1" spans="1:10">
       <c r="A136" s="3">
         <v>135</v>
       </c>
@@ -6995,7 +6995,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="139" hidden="1" spans="1:10">
+    <row r="139" ht="27" hidden="1" spans="1:10">
       <c r="A139" s="3">
         <v>138</v>
       </c>
@@ -7051,7 +7051,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="141" hidden="1" spans="1:10">
+    <row r="141" ht="27" hidden="1" spans="1:10">
       <c r="A141" s="3">
         <v>140</v>
       </c>
@@ -7107,7 +7107,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="143" hidden="1" spans="1:10">
+    <row r="143" ht="27" hidden="1" spans="1:10">
       <c r="A143" s="3">
         <v>142</v>
       </c>
@@ -7163,7 +7163,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="145" hidden="1" spans="1:10">
+    <row r="145" ht="27" hidden="1" spans="1:10">
       <c r="A145" s="3">
         <v>144</v>
       </c>
@@ -8055,7 +8055,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="174" hidden="1" spans="1:10">
+    <row r="174" ht="27" hidden="1" spans="1:10">
       <c r="A174" s="3">
         <v>173</v>
       </c>
@@ -8083,7 +8083,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="175" hidden="1" spans="1:10">
+    <row r="175" ht="27" hidden="1" spans="1:10">
       <c r="A175" s="3">
         <v>174</v>
       </c>
@@ -8111,7 +8111,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="176" hidden="1" spans="1:10">
+    <row r="176" ht="27" hidden="1" spans="1:10">
       <c r="A176" s="3">
         <v>175</v>
       </c>
@@ -8139,7 +8139,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="177" hidden="1" spans="1:10">
+    <row r="177" ht="27" hidden="1" spans="1:10">
       <c r="A177" s="3">
         <v>176</v>
       </c>
@@ -8519,7 +8519,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="190" hidden="1" spans="1:10">
+    <row r="190" ht="27" hidden="1" spans="1:10">
       <c r="A190" s="3">
         <v>189</v>
       </c>
@@ -8547,7 +8547,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="191" hidden="1" spans="1:10">
+    <row r="191" ht="27" hidden="1" spans="1:10">
       <c r="A191" s="3">
         <v>190</v>
       </c>
@@ -8575,7 +8575,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="192" hidden="1" spans="1:10">
+    <row r="192" ht="27" hidden="1" spans="1:10">
       <c r="A192" s="3">
         <v>191</v>
       </c>
@@ -8603,7 +8603,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="193" hidden="1" spans="1:10">
+    <row r="193" ht="27" hidden="1" spans="1:10">
       <c r="A193" s="3">
         <v>192</v>
       </c>
@@ -8983,7 +8983,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="206" hidden="1" spans="1:10">
+    <row r="206" ht="27" hidden="1" spans="1:10">
       <c r="A206" s="3">
         <v>205</v>
       </c>
@@ -9011,7 +9011,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="207" hidden="1" spans="1:10">
+    <row r="207" ht="27" hidden="1" spans="1:10">
       <c r="A207" s="3">
         <v>206</v>
       </c>
@@ -9039,7 +9039,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="208" hidden="1" spans="1:10">
+    <row r="208" ht="27" hidden="1" spans="1:10">
       <c r="A208" s="3">
         <v>207</v>
       </c>
@@ -9067,7 +9067,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="209" hidden="1" spans="1:10">
+    <row r="209" ht="27" hidden="1" spans="1:10">
       <c r="A209" s="3">
         <v>208</v>
       </c>
@@ -9447,7 +9447,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="222" hidden="1" spans="1:10">
+    <row r="222" ht="27" hidden="1" spans="1:10">
       <c r="A222" s="3">
         <v>221</v>
       </c>
@@ -9475,7 +9475,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="223" hidden="1" spans="1:10">
+    <row r="223" ht="27" hidden="1" spans="1:10">
       <c r="A223" s="3">
         <v>222</v>
       </c>
@@ -9503,7 +9503,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="224" hidden="1" spans="1:10">
+    <row r="224" ht="27" hidden="1" spans="1:10">
       <c r="A224" s="3">
         <v>223</v>
       </c>
@@ -9531,7 +9531,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="225" hidden="1" spans="1:10">
+    <row r="225" ht="27" hidden="1" spans="1:10">
       <c r="A225" s="3">
         <v>224</v>
       </c>
@@ -9815,7 +9815,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="235" hidden="1" spans="1:10">
+    <row r="235" ht="27" hidden="1" spans="1:10">
       <c r="A235" s="3">
         <v>234</v>
       </c>
@@ -9985,7 +9985,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="241" hidden="1" spans="1:10">
+    <row r="241" ht="27" hidden="1" spans="1:10">
       <c r="A241" s="3">
         <v>240</v>
       </c>
@@ -10155,7 +10155,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="247" hidden="1" spans="1:10">
+    <row r="247" ht="27" hidden="1" spans="1:10">
       <c r="A247" s="3">
         <v>246</v>
       </c>
@@ -10325,7 +10325,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="253" hidden="1" spans="1:10">
+    <row r="253" ht="27" hidden="1" spans="1:10">
       <c r="A253" s="3">
         <v>252</v>
       </c>
@@ -10549,7 +10549,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="261" hidden="1" spans="1:10">
+    <row r="261" ht="27" hidden="1" spans="1:10">
       <c r="A261" s="3">
         <v>260</v>
       </c>
@@ -10699,7 +10699,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="266" hidden="1" spans="1:10">
+    <row r="266" ht="27" hidden="1" spans="1:10">
       <c r="A266" s="3">
         <v>265</v>
       </c>

</xml_diff>